<commit_message>
Atualiza PDS e mapa em 2026-07-24
</commit_message>
<xml_diff>
--- a/planilha_base_mapa.xlsx
+++ b/planilha_base_mapa.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="31.109375" customWidth="1" min="1" max="1"/>
@@ -1289,6 +1289,33 @@
         </is>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>RCE Conjunto União</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>RCE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Base real do shape: SIRGAS 2000 / UTM zona 23S convertida para latitude/longitude.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1305,7 +1332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L507"/>
+  <dimension ref="A1:L518"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -24532,6 +24559,534 @@
       <c r="L507" t="inlineStr">
         <is>
           <t>As built INT Ayrton Senna enviado em 20/07/2026: PIE-01 ao PI-02, 3 pontos, 2 trechos em VCA, PVC DN200.</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>PI-44</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>PI-44</t>
+        </is>
+      </c>
+      <c r="E508" t="n">
+        <v>7398060.225</v>
+      </c>
+      <c r="F508" t="n">
+        <v>358067.987</v>
+      </c>
+      <c r="G508" t="n">
+        <v>-23.521508</v>
+      </c>
+      <c r="H508" t="n">
+        <v>-46.3902572</v>
+      </c>
+      <c r="I508" t="n">
+        <v>805.215</v>
+      </c>
+      <c r="J508" t="n">
+        <v>804.515</v>
+      </c>
+      <c r="K508" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>PI-44</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>PI-45</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>PI-45</t>
+        </is>
+      </c>
+      <c r="E509" t="n">
+        <v>7398012.158</v>
+      </c>
+      <c r="F509" t="n">
+        <v>358082.319</v>
+      </c>
+      <c r="G509" t="n">
+        <v>-23.5219433</v>
+      </c>
+      <c r="H509" t="n">
+        <v>-46.3901214</v>
+      </c>
+      <c r="I509" t="n">
+        <v>799.865</v>
+      </c>
+      <c r="J509" t="n">
+        <v>798.645</v>
+      </c>
+      <c r="K509" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>PI-45</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>PI-46</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>PI-46</t>
+        </is>
+      </c>
+      <c r="E510" t="n">
+        <v>7397944.871</v>
+      </c>
+      <c r="F510" t="n">
+        <v>358101.58</v>
+      </c>
+      <c r="G510" t="n">
+        <v>-23.5225526</v>
+      </c>
+      <c r="H510" t="n">
+        <v>-46.3899391</v>
+      </c>
+      <c r="I510" t="n">
+        <v>791.918</v>
+      </c>
+      <c r="J510" t="n">
+        <v>790.758</v>
+      </c>
+      <c r="K510" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="L510" t="inlineStr">
+        <is>
+          <t>PI-46</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>PI-47</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>PI-47</t>
+        </is>
+      </c>
+      <c r="E511" t="n">
+        <v>7397910.579</v>
+      </c>
+      <c r="F511" t="n">
+        <v>358111.228</v>
+      </c>
+      <c r="G511" t="n">
+        <v>-23.5228631</v>
+      </c>
+      <c r="H511" t="n">
+        <v>-46.3898479</v>
+      </c>
+      <c r="I511" t="n">
+        <v>785.635</v>
+      </c>
+      <c r="J511" t="n">
+        <v>784.035</v>
+      </c>
+      <c r="K511" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L511" t="inlineStr">
+        <is>
+          <t>PI-47</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>PI-48</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>PI-48</t>
+        </is>
+      </c>
+      <c r="E512" t="n">
+        <v>7397888.14</v>
+      </c>
+      <c r="F512" t="n">
+        <v>358115.915</v>
+      </c>
+      <c r="G512" t="n">
+        <v>-23.5230662</v>
+      </c>
+      <c r="H512" t="n">
+        <v>-46.3898041</v>
+      </c>
+      <c r="I512" t="n">
+        <v>780.597</v>
+      </c>
+      <c r="J512" t="n">
+        <v>779.327</v>
+      </c>
+      <c r="K512" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="L512" t="inlineStr">
+        <is>
+          <t>PI-48</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>PI-49</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>PI-49</t>
+        </is>
+      </c>
+      <c r="E513" t="n">
+        <v>7397885.895</v>
+      </c>
+      <c r="F513" t="n">
+        <v>358110.479</v>
+      </c>
+      <c r="G513" t="n">
+        <v>-23.523086</v>
+      </c>
+      <c r="H513" t="n">
+        <v>-46.3898576</v>
+      </c>
+      <c r="I513" t="n">
+        <v>780.679</v>
+      </c>
+      <c r="J513" t="n">
+        <v>779.699</v>
+      </c>
+      <c r="K513" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L513" t="inlineStr">
+        <is>
+          <t>PI-49</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>PI-50</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>PI-50</t>
+        </is>
+      </c>
+      <c r="E514" t="n">
+        <v>7397880.258</v>
+      </c>
+      <c r="F514" t="n">
+        <v>358111.652</v>
+      </c>
+      <c r="G514" t="n">
+        <v>-23.523137</v>
+      </c>
+      <c r="H514" t="n">
+        <v>-46.3898466</v>
+      </c>
+      <c r="I514" t="n">
+        <v>780.655</v>
+      </c>
+      <c r="J514" t="n">
+        <v>779.975</v>
+      </c>
+      <c r="K514" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="L514" t="inlineStr">
+        <is>
+          <t>PI-50</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>PI-52</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>PI-52</t>
+        </is>
+      </c>
+      <c r="E515" t="n">
+        <v>7397881.941</v>
+      </c>
+      <c r="F515" t="n">
+        <v>358130.022</v>
+      </c>
+      <c r="G515" t="n">
+        <v>-23.5231234</v>
+      </c>
+      <c r="H515" t="n">
+        <v>-46.3896666</v>
+      </c>
+      <c r="I515" t="n">
+        <v>780.6130000000001</v>
+      </c>
+      <c r="J515" t="n">
+        <v>779.713</v>
+      </c>
+      <c r="K515" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L515" t="inlineStr">
+        <is>
+          <t>PI-52</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>PI-53</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>PI-53</t>
+        </is>
+      </c>
+      <c r="E516" t="n">
+        <v>7397889.685</v>
+      </c>
+      <c r="F516" t="n">
+        <v>358128.139</v>
+      </c>
+      <c r="G516" t="n">
+        <v>-23.5230533</v>
+      </c>
+      <c r="H516" t="n">
+        <v>-46.3896843</v>
+      </c>
+      <c r="I516" t="n">
+        <v>780.699</v>
+      </c>
+      <c r="J516" t="n">
+        <v>779.689</v>
+      </c>
+      <c r="K516" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>PI-53</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>PV-41</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>PV-41</t>
+        </is>
+      </c>
+      <c r="E517" t="n">
+        <v>7397848.972</v>
+      </c>
+      <c r="F517" t="n">
+        <v>358119.212</v>
+      </c>
+      <c r="G517" t="n">
+        <v>-23.5234201</v>
+      </c>
+      <c r="H517" t="n">
+        <v>-46.3897755</v>
+      </c>
+      <c r="I517" t="n">
+        <v>775.5650000000001</v>
+      </c>
+      <c r="J517" t="n">
+        <v>772.015</v>
+      </c>
+      <c r="K517" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="L517" t="inlineStr">
+        <is>
+          <t>PV-41</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>PV-48.1</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>PV-48.1</t>
+        </is>
+      </c>
+      <c r="E518" t="n">
+        <v>7397886.63</v>
+      </c>
+      <c r="F518" t="n">
+        <v>358115.732</v>
+      </c>
+      <c r="G518" t="n">
+        <v>-23.5230798</v>
+      </c>
+      <c r="H518" t="n">
+        <v>-46.3898061</v>
+      </c>
+      <c r="I518" t="n">
+        <v>780.398</v>
+      </c>
+      <c r="J518" t="n">
+        <v>779.078</v>
+      </c>
+      <c r="K518" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="L518" t="inlineStr">
+        <is>
+          <t>PV-48.1</t>
         </is>
       </c>
     </row>
@@ -24546,7 +25101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R522"/>
+  <dimension ref="A1:R533"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -61700,6 +62255,732 @@
       </c>
       <c r="R522" t="n">
         <v>-46.4161627</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>CU-001</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>PI-46 - PI-47</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>PI-46</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>PI-47</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G523" t="n">
+        <v>200</v>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I523" t="n">
+        <v>35.62</v>
+      </c>
+      <c r="J523" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="K523" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="M523" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="O523" t="n">
+        <v>-23.5225526</v>
+      </c>
+      <c r="P523" t="n">
+        <v>-46.3899391</v>
+      </c>
+      <c r="Q523" t="n">
+        <v>-23.5228631</v>
+      </c>
+      <c r="R523" t="n">
+        <v>-46.3898479</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>CU-002</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>PI-47 - PI-48</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>PI-47</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>PI-48</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G524" t="n">
+        <v>200</v>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I524" t="n">
+        <v>22.92</v>
+      </c>
+      <c r="J524" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="K524" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="M524" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="O524" t="n">
+        <v>-23.5228631</v>
+      </c>
+      <c r="P524" t="n">
+        <v>-46.3898479</v>
+      </c>
+      <c r="Q524" t="n">
+        <v>-23.5230662</v>
+      </c>
+      <c r="R524" t="n">
+        <v>-46.3898041</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>CU-003</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>PI-47 - PV-48.1</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>PI-47</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>PV-48.1</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G525" t="n">
+        <v>355</v>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I525" t="n">
+        <v>24.37</v>
+      </c>
+      <c r="J525" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="K525" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="M525" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="O525" t="n">
+        <v>-23.5228631</v>
+      </c>
+      <c r="P525" t="n">
+        <v>-46.3898479</v>
+      </c>
+      <c r="Q525" t="n">
+        <v>-23.5230798</v>
+      </c>
+      <c r="R525" t="n">
+        <v>-46.3898061</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>CU-004</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>PI-48 - PV-48.1</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>PI-48</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>PV-48.1</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G526" t="n">
+        <v>200</v>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I526" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="J526" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="K526" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="M526" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="O526" t="n">
+        <v>-23.5230662</v>
+      </c>
+      <c r="P526" t="n">
+        <v>-46.3898041</v>
+      </c>
+      <c r="Q526" t="n">
+        <v>-23.5230798</v>
+      </c>
+      <c r="R526" t="n">
+        <v>-46.3898061</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>CU-005</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>PI-52 - PI-53</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>PI-52</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>PI-53</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G527" t="n">
+        <v>200</v>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I527" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="J527" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K527" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="M527" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="O527" t="n">
+        <v>-23.5231234</v>
+      </c>
+      <c r="P527" t="n">
+        <v>-46.3896666</v>
+      </c>
+      <c r="Q527" t="n">
+        <v>-23.5230533</v>
+      </c>
+      <c r="R527" t="n">
+        <v>-46.3896843</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>CU-006</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>PI-53 - PI-48</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>PI-53</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>PI-48</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G528" t="n">
+        <v>200</v>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I528" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="J528" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="K528" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="M528" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="O528" t="n">
+        <v>-23.5230533</v>
+      </c>
+      <c r="P528" t="n">
+        <v>-46.3896843</v>
+      </c>
+      <c r="Q528" t="n">
+        <v>-23.5230662</v>
+      </c>
+      <c r="R528" t="n">
+        <v>-46.3898041</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>CU-007</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>PI-49 - PV-48.1</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>PI-49</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>PV-48.1</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G529" t="n">
+        <v>200</v>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I529" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="J529" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="K529" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="M529" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="O529" t="n">
+        <v>-23.523086</v>
+      </c>
+      <c r="P529" t="n">
+        <v>-46.3898576</v>
+      </c>
+      <c r="Q529" t="n">
+        <v>-23.5230798</v>
+      </c>
+      <c r="R529" t="n">
+        <v>-46.3898061</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>CU-008</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>PI-50 - PI-49</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>PI-50</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>PI-49</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G530" t="n">
+        <v>200</v>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I530" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="J530" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="K530" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="M530" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="O530" t="n">
+        <v>-23.523137</v>
+      </c>
+      <c r="P530" t="n">
+        <v>-46.3898466</v>
+      </c>
+      <c r="Q530" t="n">
+        <v>-23.523086</v>
+      </c>
+      <c r="R530" t="n">
+        <v>-46.3898576</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>CU-009</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>PI-44 - PI-45</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>PI-44</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>PI-45</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G531" t="n">
+        <v>200</v>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I531" t="n">
+        <v>50.16</v>
+      </c>
+      <c r="J531" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K531" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="M531" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="O531" t="n">
+        <v>-23.521508</v>
+      </c>
+      <c r="P531" t="n">
+        <v>-46.3902572</v>
+      </c>
+      <c r="Q531" t="n">
+        <v>-23.5219433</v>
+      </c>
+      <c r="R531" t="n">
+        <v>-46.3901214</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>CU-010</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>PI-45 - PI-46</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>PI-45</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>PI-46</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G532" t="n">
+        <v>200</v>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I532" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="J532" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="K532" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="M532" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="O532" t="n">
+        <v>-23.5219433</v>
+      </c>
+      <c r="P532" t="n">
+        <v>-46.3901214</v>
+      </c>
+      <c r="Q532" t="n">
+        <v>-23.5225526</v>
+      </c>
+      <c r="R532" t="n">
+        <v>-46.3899391</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>conjunto_uniao</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>CU-011</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>PV-48.1 - PV-41</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>PV-48.1</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>PV-41</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G533" t="n">
+        <v>355</v>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I533" t="n">
+        <v>37.82</v>
+      </c>
+      <c r="J533" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="K533" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="M533" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="O533" t="n">
+        <v>-23.5230798</v>
+      </c>
+      <c r="P533" t="n">
+        <v>-46.3898061</v>
+      </c>
+      <c r="Q533" t="n">
+        <v>-23.5234201</v>
+      </c>
+      <c r="R533" t="n">
+        <v>-46.3897755</v>
       </c>
     </row>
   </sheetData>

</xml_diff>